<commit_message>
Add source_status field and SourceStatusEnum to SourceInformation
Adds a required source_status slot on SourceInformation, backed by a new
SourceStatusEnum (maintained_regular_updates, maintained_as_needed_updates,
not_maintained, unknown), and regenerates project artifacts + the pydantic
datamodel.

This field is referenced by the translator-ingests RIG template and the
June 2026 RIG review guidance but was not yet present in the schema, so RIGs
that populate source_status currently fail validation.
</commit_message>
<xml_diff>
--- a/project/excel/resource_ingest_guide_schema.xlsx
+++ b/project/excel/resource_ingest_guide_schema.xlsx
@@ -7,9 +7,21 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NamedThing" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ReferenceIngestGuide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ReferenceIngestGuideCollection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ReferenceIngestGuide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SupportingDataSourceInformation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SourceInformation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TermsOfUseInformation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IngestInformation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="RelevantFiles" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="IncludedContent" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FilteredContent" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FutureContentConsiderations" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TargetInformation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="EdgeType" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Qualifier" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="NodeType" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="FutureModelingConsiderations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="ProvenanceInformation" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,104 +427,655 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>primary_email</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>birth_date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>age_in_years</t>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>supporting_data_source_info</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>source_info</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>vital_status</t>
+          <t>ingest_info</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>target_info</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>provenance_info</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>infores_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>edge_type_info</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>node_type_info</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>future_considerations</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>subject_categories</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>predicates</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>object_categories</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>qualifiers</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>knowledge_level</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>agent_type</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ALIVE,DEAD,UNKNOWN"</formula1>
+          <t>primary_knowledge_sources</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>supporting_data_sources</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>aggregator_knowledge_sources</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>edge_properties</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ui_explanation</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>source_files</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"knowledge_assertion,logical_entailment,prediction,statistical_association,observation,not_provided,varies"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"manual_agent,automated_agent,computational_model,data_analysis_pipeline,text_mining_agent,image_processing_agent,manual_validation_of_automated_agent,experimental_agent,not_provided,varies"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_range</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>value_enumeration</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value_id_prefixes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>value_description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>node_category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_identifier_types</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>node_properties</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>consideration</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"spoq_pattern,predicates,qualifiers,edge_properties,node_properties,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>contributions</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>artifacts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>infores_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>terms_of_use_info</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>relevant_files</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>entries</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>infores_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>citations</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>terms_of_use_info</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>data_access_locations</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>data_provision_mechanisms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>data_formats</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>data_versioning_and_releases</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>source_status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"file_download,api_endpoint,database_dump,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"tsv,xml,csv,json,yaml,obo,protobuff,kgx,mysql,postgresql,sqlite,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"maintained_regular_updates,maintained_as_needed_updates,not_maintained,unknown"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>terms_of_use_url</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>terms_of_use_description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>license_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>license_url</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ingest_categories</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>relevant_files</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>included_content</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>filtered_content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>future_considerations</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"primary_knowledge_provider,aggregation_provider,aggregation_interpreter,supporting_data_provider,translator_knowledge_creator,ontology_provider,node_property_only_provider,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>included_records</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fields_used</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>filtered_records</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>consideration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>relevant_files</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"edge_content,node_property_content,edge_property_content,other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete #48 intent: enum form, included_content optional, additional_notes multivalued, regenerate artifacts
- Rewrite SourceStatusEnum permissible_values into valid LinkML form
  (description sub-keys) using the same 4 values
- Make IngestInformation.included_content optional
- Make all additional_notes slots multivalued (per PR description)
- Regenerate project/ artifacts + pydantic datamodel via make gen-project

Co-authored-by: Matthew Brush <mhb120@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/resource_ingest_guide_schema.xlsx
+++ b/project/excel/resource_ingest_guide_schema.xlsx
@@ -7,9 +7,21 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NamedThing" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ReferenceIngestGuide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ReferenceIngestGuideCollection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ReferenceIngestGuide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SupportingDataSourceInformation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SourceInformation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TermsOfUseInformation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IngestInformation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="RelevantFiles" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="IncludedContent" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FilteredContent" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FutureContentConsiderations" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TargetInformation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="EdgeType" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Qualifier" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="NodeType" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="FutureModelingConsiderations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="ProvenanceInformation" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,104 +427,655 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>primary_email</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>birth_date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>age_in_years</t>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>supporting_data_source_info</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>source_info</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>vital_status</t>
+          <t>ingest_info</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>target_info</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>provenance_info</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>infores_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>edge_type_info</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>node_type_info</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>future_considerations</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>subject_categories</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>predicates</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>object_categories</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>qualifiers</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>knowledge_level</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>agent_type</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ALIVE,DEAD,UNKNOWN"</formula1>
+          <t>primary_knowledge_sources</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>supporting_data_sources</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>aggregator_knowledge_sources</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>edge_properties</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ui_explanation</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>source_files</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"knowledge_assertion,logical_entailment,prediction,statistical_association,observation,not_provided,varies"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"manual_agent,automated_agent,computational_model,data_analysis_pipeline,text_mining_agent,image_processing_agent,manual_validation_of_automated_agent,experimental_agent,not_provided,varies"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_range</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>value_enumeration</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value_id_prefixes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>value_description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>node_category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_identifier_types</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>node_properties</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>consideration</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"spoq_pattern,predicates,qualifiers,edge_properties,node_properties,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>contributions</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>artifacts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>infores_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>terms_of_use_info</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>relevant_files</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>entries</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>infores_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>citations</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>terms_of_use_info</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>data_access_locations</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>data_provision_mechanisms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>data_formats</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>data_versioning_and_releases</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>source_status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"file_download,api_endpoint,database_dump,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"tsv,xml,csv,json,yaml,obo,protobuff,kgx,mysql,postgresql,sqlite,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"maintained_regular_updates,maintained_as_needed_updates,not_maintained,unknown"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>terms_of_use_url</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>terms_of_use_description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>license_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>license_url</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ingest_categories</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>relevant_files</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>included_content</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>filtered_content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>future_considerations</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>additional_notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"primary_knowledge_provider,aggregation_provider,aggregation_interpreter,supporting_data_provider,translator_knowledge_creator,ontology_provider,node_property_only_provider,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>included_records</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fields_used</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>filtered_records</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>consideration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>relevant_files</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"edge_content,node_property_content,edge_property_content,other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>